<commit_message>
feat(site): clarify dashboard sentiment displays
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/documents/narberth-zoning-classifications.xlsx
+++ b/docs/documents/narberth-zoning-classifications.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -906,7 +906,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -1998,7 +1998,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2518,7 +2518,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2570,7 +2570,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -2882,7 +2882,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3506,7 +3506,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -4442,7 +4442,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -4806,7 +4806,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -5222,7 +5222,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -5898,7 +5898,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -6522,7 +6522,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -6730,7 +6730,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -6782,7 +6782,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -6886,7 +6886,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -6938,7 +6938,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -7094,7 +7094,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -7146,7 +7146,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -7978,7 +7978,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -8758,7 +8758,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -8810,7 +8810,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -8862,7 +8862,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -9174,7 +9174,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -9226,7 +9226,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -9954,7 +9954,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -10006,7 +10006,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -10110,7 +10110,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -10474,7 +10474,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -10890,7 +10890,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -11202,7 +11202,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -11358,7 +11358,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -11670,7 +11670,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -11826,7 +11826,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -11878,7 +11878,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -11930,7 +11930,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -11982,7 +11982,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -12294,7 +12294,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -12346,7 +12346,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -12398,7 +12398,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -12450,7 +12450,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -12658,7 +12658,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -12762,7 +12762,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -12814,7 +12814,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -12918,7 +12918,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -13074,7 +13074,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -13126,7 +13126,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -13334,7 +13334,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -13490,7 +13490,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -13594,7 +13594,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -13698,7 +13698,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -13750,7 +13750,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -13906,7 +13906,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -14218,7 +14218,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -14530,7 +14530,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -14582,7 +14582,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -14738,7 +14738,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
@@ -15102,7 +15102,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
@@ -15154,7 +15154,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
@@ -15570,7 +15570,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -16298,7 +16298,7 @@
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H310" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H313" t="inlineStr">
@@ -16610,7 +16610,7 @@
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
@@ -16662,7 +16662,7 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
@@ -16766,7 +16766,7 @@
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
@@ -17234,7 +17234,7 @@
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H328" t="inlineStr">
@@ -17338,7 +17338,7 @@
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H330" t="inlineStr">
@@ -17702,7 +17702,7 @@
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H337" t="inlineStr">
@@ -17754,7 +17754,7 @@
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H338" t="inlineStr">
@@ -18014,7 +18014,7 @@
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
@@ -18170,7 +18170,7 @@
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H346" t="inlineStr">
@@ -18222,7 +18222,7 @@
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
@@ -18274,7 +18274,7 @@
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H348" t="inlineStr">
@@ -18326,7 +18326,7 @@
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H349" t="inlineStr">
@@ -18378,7 +18378,7 @@
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H350" t="inlineStr">
@@ -18430,7 +18430,7 @@
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H351" t="inlineStr">
@@ -18534,7 +18534,7 @@
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H353" t="inlineStr">
@@ -18586,7 +18586,7 @@
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H354" t="inlineStr">
@@ -18638,7 +18638,7 @@
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
@@ -18794,7 +18794,7 @@
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H358" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H359" t="inlineStr">
@@ -18950,7 +18950,7 @@
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H361" t="inlineStr">
@@ -19002,7 +19002,7 @@
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H362" t="inlineStr">
@@ -19106,7 +19106,7 @@
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H364" t="inlineStr">
@@ -19366,7 +19366,7 @@
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H369" t="inlineStr">
@@ -19574,7 +19574,7 @@
       </c>
       <c r="G373" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H373" t="inlineStr">
@@ -20094,7 +20094,7 @@
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H383" t="inlineStr">
@@ -20198,7 +20198,7 @@
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H385" t="inlineStr">
@@ -20302,7 +20302,7 @@
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H387" t="inlineStr">
@@ -20406,7 +20406,7 @@
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H389" t="inlineStr">
@@ -20458,7 +20458,7 @@
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H390" t="inlineStr">
@@ -20510,7 +20510,7 @@
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H391" t="inlineStr">
@@ -20562,7 +20562,7 @@
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H392" t="inlineStr">
@@ -21186,7 +21186,7 @@
       </c>
       <c r="G404" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H404" t="inlineStr">
@@ -21238,7 +21238,7 @@
       </c>
       <c r="G405" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H405" t="inlineStr">
@@ -21290,7 +21290,7 @@
       </c>
       <c r="G406" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H406" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H413" t="inlineStr">
@@ -21914,7 +21914,7 @@
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H418" t="inlineStr">
@@ -22018,7 +22018,7 @@
       </c>
       <c r="G420" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H420" t="inlineStr">
@@ -22330,7 +22330,7 @@
       </c>
       <c r="G426" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H426" t="inlineStr">
@@ -22538,7 +22538,7 @@
       </c>
       <c r="G430" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H430" t="inlineStr">
@@ -22642,7 +22642,7 @@
       </c>
       <c r="G432" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H432" t="inlineStr">
@@ -22694,7 +22694,7 @@
       </c>
       <c r="G433" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">
@@ -23110,7 +23110,7 @@
       </c>
       <c r="G441" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H441" t="inlineStr">
@@ -24046,7 +24046,7 @@
       </c>
       <c r="G459" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H459" t="inlineStr">
@@ -24098,7 +24098,7 @@
       </c>
       <c r="G460" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H460" t="inlineStr">
@@ -24358,7 +24358,7 @@
       </c>
       <c r="G465" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H465" t="inlineStr">
@@ -24514,7 +24514,7 @@
       </c>
       <c r="G468" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H468" t="inlineStr">
@@ -24566,7 +24566,7 @@
       </c>
       <c r="G469" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H469" t="inlineStr">
@@ -24670,7 +24670,7 @@
       </c>
       <c r="G471" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H471" t="inlineStr">
@@ -24826,7 +24826,7 @@
       </c>
       <c r="G474" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H474" t="inlineStr">
@@ -24878,7 +24878,7 @@
       </c>
       <c r="G475" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H475" t="inlineStr">
@@ -24930,7 +24930,7 @@
       </c>
       <c r="G476" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H476" t="inlineStr">
@@ -25034,7 +25034,7 @@
       </c>
       <c r="G478" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H478" t="inlineStr">
@@ -25242,7 +25242,7 @@
       </c>
       <c r="G482" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H482" t="inlineStr">
@@ -25450,7 +25450,7 @@
       </c>
       <c r="G486" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H486" t="inlineStr">
@@ -25710,7 +25710,7 @@
       </c>
       <c r="G491" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H491" t="inlineStr">
@@ -25762,7 +25762,7 @@
       </c>
       <c r="G492" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H492" t="inlineStr">
@@ -25866,7 +25866,7 @@
       </c>
       <c r="G494" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H494" t="inlineStr">
@@ -25970,7 +25970,7 @@
       </c>
       <c r="G496" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H496" t="inlineStr">
@@ -26334,7 +26334,7 @@
       </c>
       <c r="G503" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H503" t="inlineStr">
@@ -26386,7 +26386,7 @@
       </c>
       <c r="G504" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H504" t="inlineStr">
@@ -26594,7 +26594,7 @@
       </c>
       <c r="G508" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H508" t="inlineStr">
@@ -27114,7 +27114,7 @@
       </c>
       <c r="G518" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H518" t="inlineStr">
@@ -27218,7 +27218,7 @@
       </c>
       <c r="G520" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H520" t="inlineStr">
@@ -27426,7 +27426,7 @@
       </c>
       <c r="G524" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H524" t="inlineStr">
@@ -27634,7 +27634,7 @@
       </c>
       <c r="G528" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H528" t="inlineStr">
@@ -27686,7 +27686,7 @@
       </c>
       <c r="G529" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H529" t="inlineStr">
@@ -27738,7 +27738,7 @@
       </c>
       <c r="G530" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H530" t="inlineStr">
@@ -28102,7 +28102,7 @@
       </c>
       <c r="G537" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H537" t="inlineStr">
@@ -28362,7 +28362,7 @@
       </c>
       <c r="G542" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H542" t="inlineStr">
@@ -28570,7 +28570,7 @@
       </c>
       <c r="G546" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H546" t="inlineStr">
@@ -28622,7 +28622,7 @@
       </c>
       <c r="G547" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H547" t="inlineStr">
@@ -28778,7 +28778,7 @@
       </c>
       <c r="G550" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H550" t="inlineStr">
@@ -28830,7 +28830,7 @@
       </c>
       <c r="G551" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H551" t="inlineStr">
@@ -28882,7 +28882,7 @@
       </c>
       <c r="G552" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H552" t="inlineStr">
@@ -28986,7 +28986,7 @@
       </c>
       <c r="G554" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H554" t="inlineStr">
@@ -29090,7 +29090,7 @@
       </c>
       <c r="G556" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H556" t="inlineStr">
@@ -29246,7 +29246,7 @@
       </c>
       <c r="G559" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H559" t="inlineStr">
@@ -29298,7 +29298,7 @@
       </c>
       <c r="G560" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H560" t="inlineStr">
@@ -29454,7 +29454,7 @@
       </c>
       <c r="G563" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H563" t="inlineStr">
@@ -29506,7 +29506,7 @@
       </c>
       <c r="G564" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H564" t="inlineStr">
@@ -29714,7 +29714,7 @@
       </c>
       <c r="G568" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H568" t="inlineStr">
@@ -29818,7 +29818,7 @@
       </c>
       <c r="G570" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H570" t="inlineStr">
@@ -29922,7 +29922,7 @@
       </c>
       <c r="G572" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H572" t="inlineStr">
@@ -29974,7 +29974,7 @@
       </c>
       <c r="G573" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H573" t="inlineStr">
@@ -30130,7 +30130,7 @@
       </c>
       <c r="G576" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H576" t="inlineStr">
@@ -30286,7 +30286,7 @@
       </c>
       <c r="G579" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H579" t="inlineStr">
@@ -30338,7 +30338,7 @@
       </c>
       <c r="G580" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H580" t="inlineStr">
@@ -30494,7 +30494,7 @@
       </c>
       <c r="G583" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H583" t="inlineStr">
@@ -30650,7 +30650,7 @@
       </c>
       <c r="G586" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H586" t="inlineStr">
@@ -30910,7 +30910,7 @@
       </c>
       <c r="G591" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H591" t="inlineStr">
@@ -31378,7 +31378,7 @@
       </c>
       <c r="G600" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H600" t="inlineStr">
@@ -31482,7 +31482,7 @@
       </c>
       <c r="G602" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H602" t="inlineStr">
@@ -32074,7 +32074,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -32282,7 +32282,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -32386,7 +32386,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -32490,7 +32490,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -32854,7 +32854,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -33062,7 +33062,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -33478,7 +33478,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -33582,7 +33582,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -34050,7 +34050,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -34102,7 +34102,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -34154,7 +34154,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -34258,7 +34258,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -34362,7 +34362,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -34466,7 +34466,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -34518,7 +34518,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -34674,7 +34674,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -34778,7 +34778,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -34830,7 +34830,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -34934,7 +34934,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -35090,7 +35090,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -35194,7 +35194,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -35298,7 +35298,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -35402,7 +35402,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -35922,7 +35922,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -36026,7 +36026,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -36130,7 +36130,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -36390,7 +36390,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -36806,7 +36806,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -37066,7 +37066,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -37222,7 +37222,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
@@ -37482,7 +37482,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -37846,7 +37846,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -37898,7 +37898,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -38106,7 +38106,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -38314,7 +38314,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -38366,7 +38366,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -38470,7 +38470,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -38522,7 +38522,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -38678,7 +38678,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -38730,7 +38730,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -38834,7 +38834,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -39042,7 +39042,7 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -39562,7 +39562,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H150" t="inlineStr">
@@ -39926,7 +39926,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -40342,7 +40342,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -40394,7 +40394,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -40446,7 +40446,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
@@ -40498,7 +40498,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -40758,7 +40758,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -40810,7 +40810,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
@@ -41070,7 +41070,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -41538,7 +41538,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -41590,7 +41590,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -41694,7 +41694,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -42058,7 +42058,7 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
@@ -42214,7 +42214,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -42474,7 +42474,7 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
@@ -42786,7 +42786,7 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
@@ -42942,7 +42942,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -43046,7 +43046,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -43254,7 +43254,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -43410,7 +43410,7 @@
       </c>
       <c r="G224" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H224" t="inlineStr">
@@ -43462,7 +43462,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -43514,7 +43514,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -43566,7 +43566,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -43774,7 +43774,7 @@
       </c>
       <c r="G231" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H231" t="inlineStr">
@@ -43878,7 +43878,7 @@
       </c>
       <c r="G233" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H233" t="inlineStr">
@@ -43930,7 +43930,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -43982,7 +43982,7 @@
       </c>
       <c r="G235" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H235" t="inlineStr">
@@ -44034,7 +44034,7 @@
       </c>
       <c r="G236" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H236" t="inlineStr">
@@ -44242,7 +44242,7 @@
       </c>
       <c r="G240" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
@@ -44346,7 +44346,7 @@
       </c>
       <c r="G242" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -44398,7 +44398,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -44502,7 +44502,7 @@
       </c>
       <c r="G245" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -44658,7 +44658,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -44710,7 +44710,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -44918,7 +44918,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -45074,7 +45074,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -45178,7 +45178,7 @@
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -45282,7 +45282,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -45334,7 +45334,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -45490,7 +45490,7 @@
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -45802,7 +45802,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -46114,7 +46114,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -46166,7 +46166,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -46322,7 +46322,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
@@ -46686,7 +46686,7 @@
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H287" t="inlineStr">
@@ -46738,7 +46738,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
@@ -47154,7 +47154,7 @@
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
@@ -47954,7 +47954,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -48110,7 +48110,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -48266,7 +48266,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -48318,7 +48318,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -48422,7 +48422,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -48890,7 +48890,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -48994,7 +48994,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -49358,7 +49358,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -49410,7 +49410,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -49670,7 +49670,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -49826,7 +49826,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -49878,7 +49878,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -49930,7 +49930,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -49982,7 +49982,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -50034,7 +50034,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -50086,7 +50086,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -50190,7 +50190,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -50242,7 +50242,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -50294,7 +50294,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -50450,7 +50450,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -50502,7 +50502,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -50606,7 +50606,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -50658,7 +50658,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -50762,7 +50762,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -51022,7 +51022,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -51230,7 +51230,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -51750,7 +51750,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -51854,7 +51854,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -51958,7 +51958,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -52062,7 +52062,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -52114,7 +52114,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
@@ -52166,7 +52166,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -52218,7 +52218,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -52842,7 +52842,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
@@ -52894,7 +52894,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
@@ -52946,7 +52946,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
@@ -53310,7 +53310,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
@@ -53570,7 +53570,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -53674,7 +53674,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -53986,7 +53986,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -54194,7 +54194,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -54298,7 +54298,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -54350,7 +54350,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -54766,7 +54766,7 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -55702,7 +55702,7 @@
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -55754,7 +55754,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">
@@ -56014,7 +56014,7 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
@@ -56170,7 +56170,7 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
@@ -56222,7 +56222,7 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
@@ -56326,7 +56326,7 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
@@ -56482,7 +56482,7 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
@@ -56534,7 +56534,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
@@ -56586,7 +56586,7 @@
       </c>
       <c r="G173" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H173" t="inlineStr">
@@ -56690,7 +56690,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
@@ -56898,7 +56898,7 @@
       </c>
       <c r="G179" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H179" t="inlineStr">
@@ -57106,7 +57106,7 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
@@ -57366,7 +57366,7 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
@@ -57418,7 +57418,7 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
@@ -57522,7 +57522,7 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
@@ -57626,7 +57626,7 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
@@ -57990,7 +57990,7 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
@@ -58042,7 +58042,7 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
@@ -58250,7 +58250,7 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
@@ -58770,7 +58770,7 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
@@ -58874,7 +58874,7 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
@@ -59082,7 +59082,7 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
@@ -59290,7 +59290,7 @@
       </c>
       <c r="G225" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
@@ -59342,7 +59342,7 @@
       </c>
       <c r="G226" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
@@ -59394,7 +59394,7 @@
       </c>
       <c r="G227" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H227" t="inlineStr">
@@ -59758,7 +59758,7 @@
       </c>
       <c r="G234" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H234" t="inlineStr">
@@ -60018,7 +60018,7 @@
       </c>
       <c r="G239" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H239" t="inlineStr">
@@ -60226,7 +60226,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -60278,7 +60278,7 @@
       </c>
       <c r="G244" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H244" t="inlineStr">
@@ -60434,7 +60434,7 @@
       </c>
       <c r="G247" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H247" t="inlineStr">
@@ -60486,7 +60486,7 @@
       </c>
       <c r="G248" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H248" t="inlineStr">
@@ -60538,7 +60538,7 @@
       </c>
       <c r="G249" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H249" t="inlineStr">
@@ -60642,7 +60642,7 @@
       </c>
       <c r="G251" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H251" t="inlineStr">
@@ -60746,7 +60746,7 @@
       </c>
       <c r="G253" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H253" t="inlineStr">
@@ -60902,7 +60902,7 @@
       </c>
       <c r="G256" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H256" t="inlineStr">
@@ -60954,7 +60954,7 @@
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -61110,7 +61110,7 @@
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
@@ -61162,7 +61162,7 @@
       </c>
       <c r="G261" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H261" t="inlineStr">
@@ -61370,7 +61370,7 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
@@ -61474,7 +61474,7 @@
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -61578,7 +61578,7 @@
       </c>
       <c r="G269" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
@@ -61630,7 +61630,7 @@
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
@@ -61786,7 +61786,7 @@
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H273" t="inlineStr">
@@ -61942,7 +61942,7 @@
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -61994,7 +61994,7 @@
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
@@ -62150,7 +62150,7 @@
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
@@ -62306,7 +62306,7 @@
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
@@ -62566,7 +62566,7 @@
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H288" t="inlineStr">
@@ -63034,7 +63034,7 @@
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
@@ -63138,7 +63138,7 @@
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
       <c r="H299" t="inlineStr">
@@ -63717,7 +63717,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -63877,7 +63877,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -63941,7 +63941,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -64005,7 +64005,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -64261,7 +64261,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -64485,7 +64485,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -64805,7 +64805,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -64869,7 +64869,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65253,7 +65253,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -65285,7 +65285,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65317,7 +65317,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65381,7 +65381,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -65445,7 +65445,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65509,7 +65509,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65541,7 +65541,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65637,7 +65637,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65733,7 +65733,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65765,7 +65765,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -65829,7 +65829,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -66021,7 +66021,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -66085,7 +66085,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -66149,7 +66149,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -66213,7 +66213,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -66821,7 +66821,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -66885,7 +66885,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -66949,7 +66949,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -67109,7 +67109,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -67589,7 +67589,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -67813,7 +67813,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -67941,7 +67941,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -68165,7 +68165,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -68453,7 +68453,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -68485,7 +68485,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -68709,7 +68709,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -68837,7 +68837,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -68869,7 +68869,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -68933,7 +68933,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -68965,7 +68965,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -69061,7 +69061,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -69093,7 +69093,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -69157,7 +69157,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -69381,7 +69381,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -69797,7 +69797,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -70085,7 +70085,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -70405,7 +70405,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -70437,7 +70437,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -70469,7 +70469,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -70501,7 +70501,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -70757,7 +70757,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -70789,7 +70789,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -70981,7 +70981,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -71397,7 +71397,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -71429,7 +71429,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -71493,7 +71493,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -71749,7 +71749,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -71973,7 +71973,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -72165,7 +72165,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -72485,7 +72485,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -72613,7 +72613,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -72677,7 +72677,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -72901,7 +72901,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73061,7 +73061,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73093,7 +73093,7 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73125,7 +73125,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73157,7 +73157,7 @@
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73381,7 +73381,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -73477,7 +73477,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -73509,7 +73509,7 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -73541,7 +73541,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73573,7 +73573,7 @@
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73733,7 +73733,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -73829,7 +73829,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73861,7 +73861,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -73925,7 +73925,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74053,7 +74053,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74085,7 +74085,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74309,7 +74309,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74405,7 +74405,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -74469,7 +74469,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74533,7 +74533,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74565,7 +74565,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74693,7 +74693,7 @@
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -74885,7 +74885,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -75109,7 +75109,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -75141,7 +75141,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -75365,7 +75365,7 @@
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -75685,7 +75685,7 @@
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -75717,7 +75717,7 @@
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -76101,7 +76101,7 @@
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -76581,7 +76581,7 @@
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -76709,7 +76709,7 @@
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -76805,7 +76805,7 @@
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -76837,7 +76837,7 @@
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -76901,7 +76901,7 @@
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -77285,7 +77285,7 @@
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -77349,7 +77349,7 @@
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -77573,7 +77573,7 @@
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -77605,7 +77605,7 @@
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -77797,7 +77797,7 @@
       </c>
       <c r="F449" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -77925,7 +77925,7 @@
       </c>
       <c r="F453" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -77957,7 +77957,7 @@
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -77989,7 +77989,7 @@
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78021,7 +78021,7 @@
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78053,7 +78053,7 @@
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78085,7 +78085,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78213,7 +78213,7 @@
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78245,7 +78245,7 @@
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78277,7 +78277,7 @@
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78437,7 +78437,7 @@
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78469,7 +78469,7 @@
       </c>
       <c r="F470" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78565,7 +78565,7 @@
       </c>
       <c r="F473" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78597,7 +78597,7 @@
       </c>
       <c r="F474" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78661,7 +78661,7 @@
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78853,7 +78853,7 @@
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -78981,7 +78981,7 @@
       </c>
       <c r="F486" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -79365,7 +79365,7 @@
       </c>
       <c r="F498" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -79429,7 +79429,7 @@
       </c>
       <c r="F500" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -79525,7 +79525,7 @@
       </c>
       <c r="F503" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -79589,7 +79589,7 @@
       </c>
       <c r="F505" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -79621,7 +79621,7 @@
       </c>
       <c r="F506" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -79653,7 +79653,7 @@
       </c>
       <c r="F507" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -79685,7 +79685,7 @@
       </c>
       <c r="F508" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -80165,7 +80165,7 @@
       </c>
       <c r="F523" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -80197,7 +80197,7 @@
       </c>
       <c r="F524" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -80229,7 +80229,7 @@
       </c>
       <c r="F525" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -80517,7 +80517,7 @@
       </c>
       <c r="F534" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -80677,7 +80677,7 @@
       </c>
       <c r="F539" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -80741,7 +80741,7 @@
       </c>
       <c r="F541" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -80933,7 +80933,7 @@
       </c>
       <c r="F547" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -81061,7 +81061,7 @@
       </c>
       <c r="F551" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -81125,7 +81125,7 @@
       </c>
       <c r="F553" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -81157,7 +81157,7 @@
       </c>
       <c r="F554" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -81477,7 +81477,7 @@
       </c>
       <c r="F564" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -82309,7 +82309,7 @@
       </c>
       <c r="F590" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -82341,7 +82341,7 @@
       </c>
       <c r="F591" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -82565,7 +82565,7 @@
       </c>
       <c r="F598" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -82693,7 +82693,7 @@
       </c>
       <c r="F602" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -82725,7 +82725,7 @@
       </c>
       <c r="F603" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -82789,7 +82789,7 @@
       </c>
       <c r="F605" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -82917,7 +82917,7 @@
       </c>
       <c r="F609" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -82949,7 +82949,7 @@
       </c>
       <c r="F610" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -82981,7 +82981,7 @@
       </c>
       <c r="F611" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -83045,7 +83045,7 @@
       </c>
       <c r="F613" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -83173,7 +83173,7 @@
       </c>
       <c r="F617" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -83333,7 +83333,7 @@
       </c>
       <c r="F622" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -83557,7 +83557,7 @@
       </c>
       <c r="F629" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -83589,7 +83589,7 @@
       </c>
       <c r="F630" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -83653,7 +83653,7 @@
       </c>
       <c r="F632" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -83717,7 +83717,7 @@
       </c>
       <c r="F634" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -84037,7 +84037,7 @@
       </c>
       <c r="F644" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -84069,7 +84069,7 @@
       </c>
       <c r="F645" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -84197,7 +84197,7 @@
       </c>
       <c r="F649" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -84613,7 +84613,7 @@
       </c>
       <c r="F662" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -84677,7 +84677,7 @@
       </c>
       <c r="F664" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -84869,7 +84869,7 @@
       </c>
       <c r="F670" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -85029,7 +85029,7 @@
       </c>
       <c r="F675" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -85061,7 +85061,7 @@
       </c>
       <c r="F676" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -85093,7 +85093,7 @@
       </c>
       <c r="F677" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -85413,7 +85413,7 @@
       </c>
       <c r="F687" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -85605,7 +85605,7 @@
       </c>
       <c r="F693" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -85765,7 +85765,7 @@
       </c>
       <c r="F698" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -85797,7 +85797,7 @@
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -85893,7 +85893,7 @@
       </c>
       <c r="F702" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -85925,7 +85925,7 @@
       </c>
       <c r="F703" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -85957,7 +85957,7 @@
       </c>
       <c r="F704" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86021,7 +86021,7 @@
       </c>
       <c r="F706" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86085,7 +86085,7 @@
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86245,7 +86245,7 @@
       </c>
       <c r="F713" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -86277,7 +86277,7 @@
       </c>
       <c r="F714" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -86373,7 +86373,7 @@
       </c>
       <c r="F717" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86405,7 +86405,7 @@
       </c>
       <c r="F718" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86565,7 +86565,7 @@
       </c>
       <c r="F723" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86661,7 +86661,7 @@
       </c>
       <c r="F726" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -86725,7 +86725,7 @@
       </c>
       <c r="F728" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -86757,7 +86757,7 @@
       </c>
       <c r="F729" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86853,7 +86853,7 @@
       </c>
       <c r="F732" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -86949,7 +86949,7 @@
       </c>
       <c r="F735" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -86981,7 +86981,7 @@
       </c>
       <c r="F736" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>
@@ -87077,7 +87077,7 @@
       </c>
       <c r="F739" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -87173,7 +87173,7 @@
       </c>
       <c r="F742" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -87333,7 +87333,7 @@
       </c>
       <c r="F747" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -87685,7 +87685,7 @@
       </c>
       <c r="F758" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General support</t>
         </is>
       </c>
     </row>
@@ -87749,7 +87749,7 @@
       </c>
       <c r="F760" t="inlineStr">
         <is>
-          <t>General stance</t>
+          <t>General opposition</t>
         </is>
       </c>
     </row>

</xml_diff>